<commit_message>
docs: add Agreement sheet (Kraken2 vs PathSeq concordance, all 11 cohorts)
Cohort-independent aggregate table, 159 comparable samples: agreement %,
both-detected, both-negative, Kraken2-only, PathSeq-only per taxon, plus
the caveats already established in docs/pathseq_full_cohort_comparison_2026-08-23.md
(taxid mapping across PathSeq's RefSeq-81 vintage, 4A-R exclusion,
which taxa are actually well-corroborated vs. noisy).

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/neurotrophic_virus_tracking.xlsx
+++ b/docs/neurotrophic_virus_tracking.xlsx
@@ -9,7 +9,8 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="1" state="visible" r:id="rId1"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="By Sample" sheetId="2" state="visible" r:id="rId2"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="PathSeq" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="By Cohort" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Agreement" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="By Cohort" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Summary'!$A$4:$J$15</definedName>
@@ -13055,6 +13056,252 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
+  <dimension ref="A1:G17"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="32" customWidth="1" min="1" max="1"/>
+    <col width="20" customWidth="1" min="2" max="2"/>
+    <col width="14" customWidth="1" min="3" max="3"/>
+    <col width="16" customWidth="1" min="4" max="4"/>
+    <col width="16" customWidth="1" min="5" max="5"/>
+    <col width="16" customWidth="1" min="6" max="6"/>
+    <col width="16" customWidth="1" min="7" max="7"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Neurotrophic Virus Screen — Agreement (Kraken2 vs. PathSeq, all 11 cohorts)</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="3" t="inlineStr">
+        <is>
+          <t>Taxon</t>
+        </is>
+      </c>
+      <c r="B4" s="3" t="inlineStr">
+        <is>
+          <t>n (comparable samples)</t>
+        </is>
+      </c>
+      <c r="C4" s="3" t="inlineStr">
+        <is>
+          <t>Agreement %</t>
+        </is>
+      </c>
+      <c r="D4" s="3" t="inlineStr">
+        <is>
+          <t>Both detected</t>
+        </is>
+      </c>
+      <c r="E4" s="3" t="inlineStr">
+        <is>
+          <t>Both negative</t>
+        </is>
+      </c>
+      <c r="F4" s="3" t="inlineStr">
+        <is>
+          <t>Kraken2-only</t>
+        </is>
+      </c>
+      <c r="G4" s="3" t="inlineStr">
+        <is>
+          <t>PathSeq-only</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>HERV-K</t>
+        </is>
+      </c>
+      <c r="B5" t="n">
+        <v>159</v>
+      </c>
+      <c r="C5" s="4">
+        <f>(D5+E5)/B5</f>
+        <v/>
+      </c>
+      <c r="D5" t="n">
+        <v>145</v>
+      </c>
+      <c r="E5" t="n">
+        <v>12</v>
+      </c>
+      <c r="F5" t="n">
+        <v>0</v>
+      </c>
+      <c r="G5" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>HSV-1</t>
+        </is>
+      </c>
+      <c r="B6" t="n">
+        <v>159</v>
+      </c>
+      <c r="C6" s="4">
+        <f>(D6+E6)/B6</f>
+        <v/>
+      </c>
+      <c r="D6" t="n">
+        <v>10</v>
+      </c>
+      <c r="E6" t="n">
+        <v>147</v>
+      </c>
+      <c r="F6" t="n">
+        <v>0</v>
+      </c>
+      <c r="G6" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>AAV</t>
+        </is>
+      </c>
+      <c r="B7" t="n">
+        <v>159</v>
+      </c>
+      <c r="C7" s="4">
+        <f>(D7+E7)/B7</f>
+        <v/>
+      </c>
+      <c r="D7" t="n">
+        <v>1</v>
+      </c>
+      <c r="E7" t="n">
+        <v>155</v>
+      </c>
+      <c r="F7" t="n">
+        <v>0</v>
+      </c>
+      <c r="G7" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>Rhadinovirus saimiriinegamma2</t>
+        </is>
+      </c>
+      <c r="B8" t="n">
+        <v>159</v>
+      </c>
+      <c r="C8" s="4">
+        <f>(D8+E8)/B8</f>
+        <v/>
+      </c>
+      <c r="D8" t="n">
+        <v>1</v>
+      </c>
+      <c r="E8" t="n">
+        <v>136</v>
+      </c>
+      <c r="F8" t="n">
+        <v>0</v>
+      </c>
+      <c r="G8" t="n">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>Molluscum contagiosum virus</t>
+        </is>
+      </c>
+      <c r="B9" t="n">
+        <v>159</v>
+      </c>
+      <c r="C9" s="4">
+        <f>(D9+E9)/B9</f>
+        <v/>
+      </c>
+      <c r="D9" t="n">
+        <v>4</v>
+      </c>
+      <c r="E9" t="n">
+        <v>132</v>
+      </c>
+      <c r="F9" t="n">
+        <v>10</v>
+      </c>
+      <c r="G9" t="n">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>Notes:</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>- Both methods classify the same STAR-unmapped read pool per sample (Kraken2: k-mer; PathSeq: BWA alignment) -- genuinely independent methods, direct comparison is meaningful.</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>- PathSeq's reference is RefSeq 81 (2017): HSV-1 is taxid 10298 there (vs. Kraken2's 3050292, same virus pre-/post-ICTV rename); Rhadinovirus saimiriinegamma2 is 10381 there (vs. Kraken2's 3050350).</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>- Simplexvirus atelinealpha1 / paninealpha3 (the two cross-species candidates) have no identifiable PathSeq/RefSeq-81 equivalent -- not included in this table.</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>- unknown_doloromics sample 4A-R excluded from all 159 comparisons (99.3% reagent/cross-mapping contamination; see cohort_registry.md).</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>- HERV-K is the strongest result: zero Kraken2-only misses across all 159 samples, read counts track proportionally (~45-70% of Kraken2's count).</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>- Rhadinovirus and Molluscum are the weakest: most of their PathSeq-only hits are low-count and diffuse (background/cross-mapping noise), not independent confirmations -- BLAST verification recommended before trusting either method alone on these two.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="A1:L16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>

</xml_diff>